<commit_message>
updates package following mtg with genetics team
</commit_message>
<xml_diff>
--- a/create_xml_R/data-raw/metadata/project_metadata.xlsx
+++ b/create_xml_R/data-raw/metadata/project_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liz/Documents/code/JPE/jpe-genetics-edi/create_xml_R/data-raw/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB964726-3E4B-A949-93A9-6521502F0D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744AEC66-8A10-BE48-9B0B-0241EE8979A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="140" yWindow="-20120" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dataset" sheetId="1" r:id="rId1"/>
@@ -99,9 +99,6 @@
   </si>
   <si>
     <t>principal investigator</t>
-  </si>
-  <si>
-    <t>creator</t>
   </si>
   <si>
     <t>title</t>
@@ -372,6 +369,9 @@
   </si>
   <si>
     <t>genotype</t>
+  </si>
+  <si>
+    <t>creator</t>
   </si>
 </sst>
 </file>
@@ -721,7 +721,7 @@
     </row>
     <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -4750,39 +4750,39 @@
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>52</v>
-      </c>
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -16816,199 +16816,199 @@
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="C2" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E2" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" t="s">
         <v>65</v>
       </c>
-      <c r="F2" s="3"/>
-    </row>
-    <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>60</v>
+      <c r="D4" s="1" t="s">
+        <v>66</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="E4" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>91</v>
+      <c r="B10" s="1" t="s">
+        <v>80</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
+      <c r="C10" s="9" t="s">
+        <v>92</v>
       </c>
-      <c r="E3" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F3" s="3"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D10" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>67</v>
+      <c r="E10" s="12" t="s">
+        <v>64</v>
       </c>
-      <c r="E4" s="12" t="s">
-        <v>65</v>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>82</v>
       </c>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F7" s="3"/>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F8" s="3"/>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="3"/>
-    </row>
-    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C11" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>67</v>
+      <c r="D11" s="1" t="s">
+        <v>66</v>
       </c>
-      <c r="E10" s="12" t="s">
-        <v>65</v>
+      <c r="E11" s="12" t="s">
+        <v>85</v>
       </c>
-      <c r="F10" s="3"/>
-    </row>
-    <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C11" s="9" t="s">
+      <c r="C12" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="F11" s="3"/>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>95</v>
-      </c>
       <c r="D12" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F12" s="3"/>
     </row>
@@ -21000,18 +21000,18 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -22030,93 +22030,93 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="2"/>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="2"/>
+    </row>
+    <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="2"/>
+    </row>
+    <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="2"/>
-    </row>
-    <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" s="2"/>
-    </row>
-    <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="2"/>
+    </row>
+    <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="2"/>
-    </row>
-    <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="B6" s="2"/>
+    </row>
+    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="2"/>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+      <c r="B7" s="2"/>
+    </row>
+    <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="2"/>
-    </row>
-    <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="B8" s="2"/>
     </row>
     <row r="9" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="2"/>
+    </row>
+    <row r="10" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B9" s="2"/>
-    </row>
-    <row r="10" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+      <c r="B10" s="2"/>
+    </row>
+    <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B10" s="2"/>
-    </row>
-    <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="B11" s="2"/>
     </row>
     <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="2"/>
+    </row>
+    <row r="13" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B12" s="2"/>
-    </row>
-    <row r="13" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+      <c r="B13" s="2"/>
+    </row>
+    <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B13" s="2"/>
-    </row>
-    <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>100</v>
-      </c>
       <c r="B14" s="2"/>
     </row>
     <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B15" s="2"/>
     </row>
@@ -25090,24 +25090,24 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>26</v>
-      </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -32136,7 +32136,7 @@
         <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>9</v>
@@ -40159,19 +40159,19 @@
   <sheetData>
     <row r="1" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>32</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -46212,18 +46212,18 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="B2" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -50251,30 +50251,30 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>42</v>
-      </c>
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B2" s="12">
         <v>-122.52526</v>
@@ -50289,10 +50289,10 @@
         <v>38.573937999999998</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>

</xml_diff>